<commit_message>
feat(F-NAR-019): TREE-AUT-036 polish L'oiseau de papier et le sac rouge de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-036.xlsx
+++ b/stories/arbres/TREE-AUT-036.xlsx
@@ -2562,17 +2562,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -2732,7 +2732,7 @@
         <is>
           <t>narrateur|Sarah pose le ballon, sans frapper.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -2759,17 +2759,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Le banc du parc est frais, strié. Sarah y pose le sac, ouvert. Le ballon reste dans le sable, loin. Je pourrais le pousser. Elle retient sa main. Personne ne dit le geste. Elle regarde la virgule bleue. Un grain tombe, tout seul. L'aile se déplie, sans elle. Il a choisi le bois, on dirait. Il s'ouvre. Le cuir du ballon a du sable, au loin.</t>
+          <t>Le banc du parc est frais, strié. Sarah y pose le sac, ouvert. Le ballon reste dans le sable, loin. Je pourrais le pousser. Elle retient sa main. Le banc ne dit rien. Elle regarde la virgule bleue. Un grain tombe, tout seul. L'aile se déplie, sans elle. Il a choisi le bois, on dirait. Il s'ouvre. Le cuir du ballon a du sable, au loin.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;banc&lt;/emphasis&gt; du parc est frais, strié. Sarah y pose le sac, ouvert. Le ballon reste dans le sable, loin. Je pourrais le pousser. Elle retient sa main. Personne ne dit le geste. Elle regarde la virgule bleue. Un grain tombe, tout seul. L'aile se déplie, sans elle. Il a choisi le bois, on dirait. Il s'ouvre. Le cuir du ballon a du sable, au loin.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;banc&lt;/emphasis&gt; du parc est frais, strié. Sarah y pose le sac, ouvert. Le ballon reste dans le sable, loin. Je pourrais le pousser. Elle retient sa main. Le banc ne dit rien. Elle regarde la virgule bleue. Un grain tombe, tout seul. L'aile se déplie, sans elle. Il a choisi le bois, on dirait. Il s'ouvre. Le cuir du ballon a du sable, au loin.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;banc&lt;/emphasis&gt; du parc est frais, strié. Sarah y pose le sac, ouvert. Le ballon reste dans le sable, loin. Je pourrais le pousser. Elle retient sa main. Personne ne dit le geste. Elle regarde la virgule bleue. Un grain tombe, tout seul. L'aile se déplie, sans elle. Il a choisi le bois, on dirait. Il s'ouvre. Le cuir du ballon a du sable, au loin. [pause]</t>
+          <t>Le &lt;emphasis&gt;banc&lt;/emphasis&gt; du parc est frais, strié. Sarah y pose le sac, ouvert. Le ballon reste dans le sable, loin. Je pourrais le pousser. Elle retient sa main. Le banc ne dit rien. Elle regarde la virgule bleue. Un grain tombe, tout seul. L'aile se déplie, sans elle. Il a choisi le bois, on dirait. Il s'ouvre. Le cuir du ballon a du sable, au loin. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2908,7 +2908,7 @@
 narrateur|Le ballon reste dans le sable, loin.
 enfant-f|Je pourrais le pousser.
 narrateur|Elle retient sa main.
-narrateur|Personne ne dit le geste.
+narrateur|Le banc ne dit rien.
 narrateur|Elle regarde la virgule bleue.
 narrateur|Un grain tombe, tout seul.
 narrateur|L'aile se déplie, sans elle.
@@ -3131,17 +3131,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>La grille du parc est verte, froide. Sarah tient le sac près des barres. Le ballon roule, presque contre. Je pourrais le caler là. Elle recule le cuir, nette. Le vent passe entre deux barres. La virgule bleue se tourne vers lui. L'oiseau penche, sans main. Le vent de la grille, pas celui du ballon. Il a compris le trou. Une feuille coincée tremble, puis se tait. Le sac reste ouvert, contre rien.</t>
+          <t>La grille du parc est verte, froide. Sarah tient le sac près des barres. Le ballon roule, presque contre. Je pourrais le caler là. Elle recule le cuir, nette. Le vent passe entre deux barres. La virgule bleue se tourne vers lui. L'oiseau penche, sans main. Le vent de la grille, pas celui du ballon. Il a vu le trou. Une feuille coincée tremble, puis se tait. Le sac reste ouvert, contre rien.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;grille&lt;/emphasis&gt; du parc est verte, froide. Sarah tient le sac près des barres. Le ballon roule, presque contre. Je pourrais le caler là. Elle recule le cuir, nette. Le vent passe entre deux barres. La virgule bleue se tourne vers lui. L'oiseau penche, sans main. Le vent de la grille, pas celui du ballon. Il a compris le trou. Une feuille coincée tremble, puis se tait. Le sac reste ouvert, contre rien.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;grille&lt;/emphasis&gt; du parc est verte, froide. Sarah tient le sac près des barres. Le ballon roule, presque contre. Je pourrais le caler là. Elle recule le cuir, nette. Le vent passe entre deux barres. La virgule bleue se tourne vers lui. L'oiseau penche, sans main. Le vent de la grille, pas celui du ballon. Il a vu le trou. Une feuille coincée tremble, puis se tait. Le sac reste ouvert, contre rien.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;grille&lt;/emphasis&gt; du parc est verte, froide. Sarah tient le sac près des barres. Le ballon roule, presque contre. Je pourrais le caler là. Elle recule le cuir, nette. Le vent passe entre deux barres. La virgule bleue se tourne vers lui. L'oiseau penche, sans main. Le vent de la grille, pas celui du ballon. Il a compris le trou. Une feuille coincée tremble, puis se tait. Le sac reste ouvert, contre rien. [pause]</t>
+          <t>La &lt;emphasis&gt;grille&lt;/emphasis&gt; du parc est verte, froide. Sarah tient le sac près des barres. Le ballon roule, presque contre. Je pourrais le caler là. Elle recule le cuir, nette. Le vent passe entre deux barres. La virgule bleue se tourne vers lui. L'oiseau penche, sans main. Le vent de la grille, pas celui du ballon. Il a vu le trou. Une feuille coincée tremble, puis se tait. Le sac reste ouvert, contre rien. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3284,7 +3284,7 @@
 narrateur|La virgule bleue se tourne vers lui.
 narrateur|L'oiseau penche, sans main.
 maman|Le vent de la grille, pas celui du ballon.
-enfant-f|Il a compris le trou.
+enfant-f|Il a vu le trou.
 narrateur|Une feuille coincée tremble, puis se tait.
 narrateur|Le sac reste ouvert, contre rien.</t>
         </is>
@@ -4067,17 +4067,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -4237,7 +4237,7 @@
         <is>
           <t>narrateur|Sarah pose le seau, sans verser.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -5195,17 +5195,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent, une pétale au bord du tissu. Tu raconteras le moment difficile ? Surtout quand j'ai voulu verser. L'arbre n'avait pas besoin du seau. Sarah pose le sac au pied du lit. Les sangles du sac sentent le bois, un peu.</t>
+          <t>Ils rentrent, une pétale au bord du tissu. Tu raconteras le moment difficile ? Surtout quand j'ai voulu verser. L'arbre n'avait pas besoin du seau. Sarah pose le sac au pied du lit. Les sangles du sac sentent la feuille, un peu.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent, une pétale au bord du tissu. Tu raconteras le moment difficile ? Surtout quand j'ai voulu verser. L'arbre n'avait pas besoin du seau. Sarah pose le sac au pied du lit. Les sangles du sac sentent le bois, un peu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent, une pétale au bord du tissu. Tu raconteras le moment difficile ? Surtout quand j'ai voulu verser. L'arbre n'avait pas besoin du seau. Sarah pose le sac au pied du lit. Les sangles du sac sentent la feuille, un peu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent, une pétale au bord du tissu. Tu raconteras le moment difficile ? Surtout quand j'ai voulu verser. L'arbre n'avait pas besoin du seau. Sarah pose le sac au pied du lit. Les sangles du sac sentent le bois, un peu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent, une pétale au bord du tissu. Tu raconteras le moment difficile ? Surtout quand j'ai voulu verser. L'arbre n'avait pas besoin du seau. Sarah pose le sac au pied du lit. Les sangles du sac sentent la feuille, un peu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5348,7 +5348,7 @@
 enfant-f|Surtout quand j'ai voulu verser.
 maman|L'arbre n'avait pas besoin du seau.
 narrateur|Sarah pose le sac au pied du lit.
-narrateur|Les sangles du sac sentent le bois, un peu.</t>
+narrateur|Les sangles du sac sentent la feuille, un peu.</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr">
@@ -5572,17 +5572,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -5742,7 +5742,7 @@
         <is>
           <t>narrateur|Sarah pose le doudou, sans serrer.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -7837,17 +7837,17 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -8007,7 +8007,7 @@
         <is>
           <t>narrateur|Sarah pose le ballon, sans frapper.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -9342,17 +9342,17 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -9512,7 +9512,7 @@
         <is>
           <t>narrateur|Sarah pose le seau, sans verser.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -10847,17 +10847,17 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -11017,7 +11017,7 @@
         <is>
           <t>narrateur|Sarah pose le doudou, sans serrer.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -11603,17 +11603,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent, une goutte sèche sur le gris. Tu raconteras le moment difficile ? Surtout le tapis de pente. La grille a soufflé, sans étouffer. Sarah pose le sac, un peu ouvert. Le seau pose son ombre ronde sur le tapis.</t>
+          <t>Ils rentrent, une goutte sèche sur le gris. Tu raconteras le moment difficile ? Surtout le tapis de pente. La grille a soufflé, sans étouffer. Sarah pose le sac, un peu ouvert. L'oreille du doudou garde une goutte de métal.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent, une goutte sèche sur le gris. Tu raconteras le moment difficile ? Surtout le tapis de pente. La &lt;emphasis level="moderate"&gt;grille&lt;/emphasis&gt; a soufflé, sans étouffer. Sarah pose le sac, un peu ouvert. Le seau pose son ombre ronde sur le tapis.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent, une goutte sèche sur le gris. Tu raconteras le moment difficile ? Surtout le tapis de pente. La &lt;emphasis level="moderate"&gt;grille&lt;/emphasis&gt; a soufflé, sans étouffer. Sarah pose le sac, un peu ouvert. L'oreille du doudou garde une goutte de métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent, une goutte sèche sur le gris. Tu raconteras le moment difficile ? Surtout le tapis de pente. La &lt;emphasis&gt;grille&lt;/emphasis&gt; a soufflé, sans étouffer. Sarah pose le sac, un peu ouvert. Le seau pose son ombre ronde sur le tapis.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent, une goutte sèche sur le gris. Tu raconteras le moment difficile ? Surtout le tapis de pente. La &lt;emphasis&gt;grille&lt;/emphasis&gt; a soufflé, sans étouffer. Sarah pose le sac, un peu ouvert. L'oreille du doudou garde une goutte de métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11756,7 +11756,7 @@
 enfant-f|Surtout le tapis de pente.
 maman|La grille a soufflé, sans étouffer.
 narrateur|Sarah pose le sac, un peu ouvert.
-narrateur|Le seau pose son ombre ronde sur le tapis.</t>
+narrateur|L'oreille du doudou garde une goutte de métal.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr">
@@ -11975,17 +11975,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent, un toit de feuilles dans la tête. Tu raconteras le moment difficile ? Surtout le nœud trop haut. La branche tenait, sans doudou. Sarah pose le sac au pied du lit. Le ballon s'endort contre les sangles molles.</t>
+          <t>Ils rentrent, un toit de feuilles dans la tête. Tu raconteras le moment difficile ? Surtout le nœud trop haut. La branche tenait, sans doudou. Sarah pose le sac au pied du lit. Une pétale sèche sur l'oreille du doudou.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent, un toit de feuilles dans la tête. Tu raconteras le moment difficile ? Surtout le nœud trop haut. La branche tenait, sans doudou. Sarah pose le sac au pied du lit. Le ballon s'endort contre les sangles molles.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent, un toit de feuilles dans la tête. Tu raconteras le moment difficile ? Surtout le nœud trop haut. La branche tenait, sans doudou. Sarah pose le sac au pied du lit. Une pétale sèche sur l'oreille du doudou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent, un toit de feuilles dans la tête. Tu raconteras le moment difficile ? Surtout le nœud trop haut. La branche tenait, sans doudou. Sarah pose le sac au pied du lit. Le ballon s'endort contre les sangles molles.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent, un toit de feuilles dans la tête. Tu raconteras le moment difficile ? Surtout le nœud trop haut. La branche tenait, sans doudou. Sarah pose le sac au pied du lit. Une pétale sèche sur l'oreille du doudou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12128,7 +12128,7 @@
 enfant-f|Surtout le nœud trop haut.
 maman|La branche tenait, sans doudou.
 narrateur|Sarah pose le sac au pied du lit.
-narrateur|Le ballon s'endort contre les sangles molles.</t>
+narrateur|Une pétale sèche sur l'oreille du doudou.</t>
         </is>
       </c>
       <c r="AX59" t="inlineStr">
@@ -13112,17 +13112,17 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le ballon, sans frapper. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -13282,7 +13282,7 @@
         <is>
           <t>narrateur|Sarah pose le ballon, sans frapper.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -13496,17 +13496,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent, la chaîne loin derrière. Tu raconteras le moment difficile ? Surtout le tic sur le sac. Le banc n'a pas tapé. Sarah pose le sac au pied du lit. Une pétale sèche sur le rebord, près du livre.</t>
+          <t>Ils rentrent, la chaîne loin derrière. Tu raconteras le moment difficile ? Surtout le tic sur le sac. Le banc n'a pas tapé. Sarah pose le sac au pied du lit. Le ballon s'endort contre les sangles molles.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent, la chaîne loin derrière. Tu raconteras le moment difficile ? Surtout le tic sur le sac. Le &lt;emphasis level="moderate"&gt;banc&lt;/emphasis&gt; n'a pas tapé. Sarah pose le sac au pied du lit. Une pétale sèche sur le rebord, près du livre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent, la chaîne loin derrière. Tu raconteras le moment difficile ? Surtout le tic sur le sac. Le &lt;emphasis level="moderate"&gt;banc&lt;/emphasis&gt; n'a pas tapé. Sarah pose le sac au pied du lit. Le ballon s'endort contre les sangles molles.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent, la chaîne loin derrière. Tu raconteras le moment difficile ? Surtout le tic sur le sac. Le &lt;emphasis&gt;banc&lt;/emphasis&gt; n'a pas tapé. Sarah pose le sac au pied du lit. Une pétale sèche sur le rebord, près du livre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent, la chaîne loin derrière. Tu raconteras le moment difficile ? Surtout le tic sur le sac. Le &lt;emphasis&gt;banc&lt;/emphasis&gt; n'a pas tapé. Sarah pose le sac au pied du lit. Le ballon s'endort contre les sangles molles.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13649,7 +13649,7 @@
 enfant-f|Surtout le tic sur le sac.
 maman|Le banc n'a pas tapé.
 narrateur|Sarah pose le sac au pied du lit.
-narrateur|Une pétale sèche sur le rebord, près du livre.</t>
+narrateur|Le ballon s'endort contre les sangles molles.</t>
         </is>
       </c>
       <c r="AX67" t="inlineStr">
@@ -14617,17 +14617,17 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le seau, sans verser. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -14787,7 +14787,7 @@
         <is>
           <t>narrateur|Sarah pose le seau, sans verser.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -16122,17 +16122,17 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+          <t>Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où l'oiseau peut-il s'ouvrir tout seul ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Sarah pose le doudou, sans serrer. Le banc, la grille, ou le cerisier ? Où poses-tu le sac, ouvert ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -16292,7 +16292,7 @@
         <is>
           <t>narrateur|Sarah pose le doudou, sans serrer.
 papa|Le banc, la grille, ou le cerisier ?
-maman|Où l'oiseau peut-il s'ouvrir tout seul ?</t>
+maman|Où poses-tu le sac, ouvert ?</t>
         </is>
       </c>
     </row>
@@ -17429,7 +17429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17542,6 +17542,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>